<commit_message>
Created Scrolly-Telling test page.
</commit_message>
<xml_diff>
--- a/Slow Reveal Recreations/hull-house-nationalities/polygons.xlsx
+++ b/Slow Reveal Recreations/hull-house-nationalities/polygons.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gvsu365-my.sharepoint.com/personal/s_cousilou_gvsu_edu/Documents/GVSU/Work/GA Position/Data Literacy/Visualization Recreations/Hull Houses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="578" documentId="13_ncr:1_{A993E112-2CB7-4C56-9B97-33A6DEC34B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A4ED656-C432-4863-8E2E-250C12CA12AB}"/>
+  <xr:revisionPtr revIDLastSave="706" documentId="13_ncr:1_{A993E112-2CB7-4C56-9B97-33A6DEC34B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4794D97B-B955-41A7-BB10-54AB01E1E61A}"/>
   <bookViews>
-    <workbookView xWindow="43335" yWindow="0" windowWidth="9810" windowHeight="14745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="750" windowWidth="19440" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="polygons" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="25">
   <si>
     <t>x1</t>
   </si>
@@ -163,10 +163,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -432,10 +428,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A219D47-767B-4462-B7A2-6ADD9456001C}">
-  <dimension ref="A1:J183"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J200"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -467,7 +463,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>35.58</v>
       </c>
@@ -499,7 +495,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>43.51</v>
       </c>
@@ -531,7 +527,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>44.68</v>
       </c>
@@ -563,7 +559,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>43.51</v>
       </c>
@@ -595,7 +591,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>44.07</v>
       </c>
@@ -627,7 +623,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>44.68</v>
       </c>
@@ -659,7 +655,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>44.07</v>
       </c>
@@ -691,7 +687,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>45.87</v>
       </c>
@@ -723,7 +719,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>46.38</v>
       </c>
@@ -755,7 +751,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>46.38</v>
       </c>
@@ -787,7 +783,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>46.38</v>
       </c>
@@ -819,7 +815,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>47.05</v>
       </c>
@@ -851,7 +847,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>47.05</v>
       </c>
@@ -883,7 +879,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>47.49</v>
       </c>
@@ -915,7 +911,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>47.49</v>
       </c>
@@ -947,7 +943,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>47.49</v>
       </c>
@@ -979,7 +975,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>47.49</v>
       </c>
@@ -1011,7 +1007,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>48.12</v>
       </c>
@@ -1043,7 +1039,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>48.12</v>
       </c>
@@ -1075,7 +1071,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>48.72</v>
       </c>
@@ -1107,7 +1103,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>49.31</v>
       </c>
@@ -1139,7 +1135,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>50.69</v>
       </c>
@@ -1171,7 +1167,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>49.31</v>
       </c>
@@ -1203,7 +1199,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>50.69</v>
       </c>
@@ -1235,7 +1231,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>50.69</v>
       </c>
@@ -1267,7 +1263,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>50.98</v>
       </c>
@@ -1299,7 +1295,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>49.31</v>
       </c>
@@ -1335,7 +1331,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>49.72</v>
       </c>
@@ -1371,7 +1367,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>50.99</v>
       </c>
@@ -1407,7 +1403,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>40.11</v>
       </c>
@@ -1439,7 +1435,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>40.619999999999997</v>
       </c>
@@ -1471,7 +1467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>40.619999999999997</v>
       </c>
@@ -1507,7 +1503,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>41.22</v>
       </c>
@@ -1543,7 +1539,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>41.22</v>
       </c>
@@ -1579,7 +1575,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>41.22</v>
       </c>
@@ -1615,7 +1611,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>41.79</v>
       </c>
@@ -1651,7 +1647,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>42.35</v>
       </c>
@@ -1687,7 +1683,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>42.92</v>
       </c>
@@ -1723,7 +1719,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>42.92</v>
       </c>
@@ -1759,7 +1755,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>42.92</v>
       </c>
@@ -1795,7 +1791,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>42.92</v>
       </c>
@@ -1831,7 +1827,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>43.51</v>
       </c>
@@ -1867,7 +1863,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43.51</v>
       </c>
@@ -1903,7 +1899,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44.07</v>
       </c>
@@ -1939,7 +1935,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>44.68</v>
       </c>
@@ -1975,7 +1971,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>44.68</v>
       </c>
@@ -2011,7 +2007,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>45.14</v>
       </c>
@@ -2047,7 +2043,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>45.14</v>
       </c>
@@ -2083,7 +2079,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49.74</v>
       </c>
@@ -2119,7 +2115,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50.49</v>
       </c>
@@ -2155,7 +2151,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>3.79</v>
       </c>
@@ -2191,7 +2187,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>7.29</v>
       </c>
@@ -2227,7 +2223,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>9.74</v>
       </c>
@@ -2263,7 +2259,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>11.59</v>
       </c>
@@ -2299,7 +2295,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>12.73</v>
       </c>
@@ -2335,7 +2331,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>13.39</v>
       </c>
@@ -2371,7 +2367,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>13.9</v>
       </c>
@@ -2407,7 +2403,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>15.31</v>
       </c>
@@ -2443,7 +2439,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>15.31</v>
       </c>
@@ -2479,7 +2475,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>16.440000000000001</v>
       </c>
@@ -2515,7 +2511,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>16.97</v>
       </c>
@@ -2551,7 +2547,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>18.86</v>
       </c>
@@ -2587,7 +2583,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>18.86</v>
       </c>
@@ -2623,7 +2619,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>20.91</v>
       </c>
@@ -2659,7 +2655,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>22.5</v>
       </c>
@@ -2695,7 +2691,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>22.5</v>
       </c>
@@ -2731,7 +2727,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>23.14</v>
       </c>
@@ -2767,7 +2763,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>25.28</v>
       </c>
@@ -2803,7 +2799,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>25.98</v>
       </c>
@@ -2839,7 +2835,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>25.98</v>
       </c>
@@ -2875,7 +2871,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>25.98</v>
       </c>
@@ -2911,7 +2907,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>26.72</v>
       </c>
@@ -2947,7 +2943,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>26.72</v>
       </c>
@@ -2983,7 +2979,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>26.72</v>
       </c>
@@ -3019,7 +3015,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>26.72</v>
       </c>
@@ -3055,7 +3051,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>3.79</v>
       </c>
@@ -3091,7 +3087,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>7.02</v>
       </c>
@@ -3127,7 +3123,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>11.84</v>
       </c>
@@ -3163,7 +3159,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>26.75</v>
       </c>
@@ -3199,7 +3195,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>26.75</v>
       </c>
@@ -3235,7 +3231,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>26.75</v>
       </c>
@@ -3271,7 +3267,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>26.75</v>
       </c>
@@ -3307,7 +3303,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>26.75</v>
       </c>
@@ -3343,7 +3339,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>28.84</v>
       </c>
@@ -3379,7 +3375,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>29.18</v>
       </c>
@@ -3415,7 +3411,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>29.18</v>
       </c>
@@ -3451,7 +3447,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>29.18</v>
       </c>
@@ -3487,7 +3483,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>29.6</v>
       </c>
@@ -3523,7 +3519,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>29.6</v>
       </c>
@@ -3559,7 +3555,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>29.6</v>
       </c>
@@ -3595,7 +3591,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>30.33</v>
       </c>
@@ -3631,7 +3627,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>31.73</v>
       </c>
@@ -3667,7 +3663,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>31.73</v>
       </c>
@@ -3703,7 +3699,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>31.73</v>
       </c>
@@ -3739,7 +3735,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>31.73</v>
       </c>
@@ -3775,7 +3771,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>32.43</v>
       </c>
@@ -3811,7 +3807,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>33.14</v>
       </c>
@@ -3847,7 +3843,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>33.840000000000003</v>
       </c>
@@ -3883,7 +3879,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>33.840000000000003</v>
       </c>
@@ -3919,7 +3915,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>33.840000000000003</v>
       </c>
@@ -3955,7 +3951,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>34.53</v>
       </c>
@@ -3991,7 +3987,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>34.53</v>
       </c>
@@ -4027,7 +4023,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>34.53</v>
       </c>
@@ -4063,7 +4059,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>35.270000000000003</v>
       </c>
@@ -4099,7 +4095,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>35.97</v>
       </c>
@@ -4135,7 +4131,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>35.97</v>
       </c>
@@ -4171,7 +4167,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>35.97</v>
       </c>
@@ -4207,7 +4203,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>35.97</v>
       </c>
@@ -4243,7 +4239,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>35.97</v>
       </c>
@@ -4279,7 +4275,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>35.97</v>
       </c>
@@ -4315,7 +4311,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>37.47</v>
       </c>
@@ -4351,7 +4347,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>38.1</v>
       </c>
@@ -4387,7 +4383,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>38.1</v>
       </c>
@@ -4423,7 +4419,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>38.82</v>
       </c>
@@ -4459,7 +4455,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>39.53</v>
       </c>
@@ -4495,7 +4491,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>39.53</v>
       </c>
@@ -4531,7 +4527,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>39.53</v>
       </c>
@@ -4567,7 +4563,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>40.26</v>
       </c>
@@ -4603,7 +4599,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>40.26</v>
       </c>
@@ -4639,7 +4635,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>40.26</v>
       </c>
@@ -4675,7 +4671,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>40.26</v>
       </c>
@@ -4711,7 +4707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>40.26</v>
       </c>
@@ -4747,7 +4743,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>40.26</v>
       </c>
@@ -4783,7 +4779,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>41.62</v>
       </c>
@@ -4819,7 +4815,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>42.25</v>
       </c>
@@ -4855,7 +4851,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>42.25</v>
       </c>
@@ -4891,7 +4887,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>42.98</v>
       </c>
@@ -4927,7 +4923,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>42.98</v>
       </c>
@@ -4963,7 +4959,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>42.98</v>
       </c>
@@ -4999,7 +4995,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>43.67</v>
       </c>
@@ -5035,7 +5031,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>43.67</v>
       </c>
@@ -5071,7 +5067,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>43.67</v>
       </c>
@@ -5107,7 +5103,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>44.43</v>
       </c>
@@ -5143,7 +5139,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>44.43</v>
       </c>
@@ -5179,7 +5175,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>44.43</v>
       </c>
@@ -5215,7 +5211,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>44.43</v>
       </c>
@@ -5251,7 +5247,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>44.43</v>
       </c>
@@ -5287,7 +5283,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>45.09</v>
       </c>
@@ -5323,7 +5319,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>46.59</v>
       </c>
@@ -5359,7 +5355,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>46.59</v>
       </c>
@@ -5395,7 +5391,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>47.28</v>
       </c>
@@ -5431,7 +5427,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>47.28</v>
       </c>
@@ -5467,7 +5463,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>47.28</v>
       </c>
@@ -5503,7 +5499,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>47.28</v>
       </c>
@@ -5539,7 +5535,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>48.01</v>
       </c>
@@ -5575,7 +5571,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>48.01</v>
       </c>
@@ -5611,7 +5607,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>48.01</v>
       </c>
@@ -5647,7 +5643,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>48.01</v>
       </c>
@@ -5683,7 +5679,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>48.01</v>
       </c>
@@ -5719,7 +5715,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>48.71</v>
       </c>
@@ -5755,7 +5751,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>48.71</v>
       </c>
@@ -5791,7 +5787,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>49.41</v>
       </c>
@@ -5827,7 +5823,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>51.35</v>
       </c>
@@ -5863,7 +5859,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>49.41</v>
       </c>
@@ -5899,7 +5895,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>49.41</v>
       </c>
@@ -5935,7 +5931,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>49.41</v>
       </c>
@@ -5971,7 +5967,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>49.41</v>
       </c>
@@ -6007,7 +6003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>49.41</v>
       </c>
@@ -6043,7 +6039,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>50.54</v>
       </c>
@@ -6079,7 +6075,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>49.41</v>
       </c>
@@ -6115,7 +6111,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>49.41</v>
       </c>
@@ -6151,7 +6147,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>28.84</v>
       </c>
@@ -6184,10 +6180,10 @@
         <v>6.1</v>
       </c>
       <c r="J163" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>29.51</v>
       </c>
@@ -6223,7 +6219,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>28.84</v>
       </c>
@@ -6259,7 +6255,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>30.1</v>
       </c>
@@ -6295,309 +6291,975 @@
         <v>12</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>33.86</v>
+      </c>
+      <c r="B167">
+        <v>24.65</v>
+      </c>
       <c r="C167">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>33.86</v>
+      </c>
+      <c r="D167">
+        <v>21.93</v>
+      </c>
+      <c r="E167">
+        <v>34.549999999999997</v>
       </c>
       <c r="F167">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G167">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>34.549999999999997</v>
       </c>
       <c r="H167">
         <f t="shared" si="27"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I167">
+        <v>6.1</v>
+      </c>
+      <c r="J167" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>38.83</v>
+      </c>
+      <c r="B168">
+        <v>24.65</v>
+      </c>
       <c r="C168">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>38.83</v>
+      </c>
+      <c r="D168">
+        <v>21.93</v>
+      </c>
+      <c r="E168">
+        <v>39.549999999999997</v>
       </c>
       <c r="F168">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G168">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>39.549999999999997</v>
       </c>
       <c r="H168">
         <f t="shared" si="27"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I168">
+        <v>6.1</v>
+      </c>
+      <c r="J168" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>42.37</v>
+      </c>
+      <c r="B169">
+        <v>24.65</v>
+      </c>
       <c r="C169">
         <f t="shared" ref="C169:C183" si="28">A169</f>
-        <v>0</v>
+        <v>42.37</v>
+      </c>
+      <c r="D169">
+        <v>21.93</v>
+      </c>
+      <c r="E169">
+        <v>43.7</v>
       </c>
       <c r="F169">
         <f t="shared" ref="F169:F183" si="29">D169</f>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G169">
         <f t="shared" ref="G169:G183" si="30">E169</f>
-        <v>0</v>
+        <v>43.7</v>
       </c>
       <c r="H169">
         <f t="shared" ref="H169:H183" si="31">B169</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I169">
+        <v>6.1</v>
+      </c>
+      <c r="J169" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>45.75</v>
+      </c>
+      <c r="B170">
+        <v>23.87</v>
+      </c>
       <c r="C170">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>45.75</v>
+      </c>
+      <c r="D170">
+        <v>21.93</v>
+      </c>
+      <c r="E170">
+        <v>46.61</v>
       </c>
       <c r="F170">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G170">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>46.61</v>
       </c>
       <c r="H170">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.35">
+        <v>23.87</v>
+      </c>
+      <c r="I170">
+        <v>6.1</v>
+      </c>
+      <c r="J170" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>45.86</v>
+      </c>
+      <c r="B171">
+        <v>24.65</v>
+      </c>
       <c r="C171">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>45.86</v>
+      </c>
+      <c r="D171">
+        <v>23.87</v>
+      </c>
+      <c r="E171">
+        <v>46.61</v>
       </c>
       <c r="F171">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>23.87</v>
       </c>
       <c r="G171">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>46.61</v>
       </c>
       <c r="H171">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I171">
+        <v>6.1</v>
+      </c>
+      <c r="J171" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>46.61</v>
+      </c>
+      <c r="B172">
+        <v>24.65</v>
+      </c>
       <c r="C172">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>46.61</v>
+      </c>
+      <c r="D172">
+        <v>23.44</v>
+      </c>
+      <c r="E172">
+        <v>47.25</v>
       </c>
       <c r="F172">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>23.44</v>
       </c>
       <c r="G172">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>47.25</v>
       </c>
       <c r="H172">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I172">
+        <v>6.1</v>
+      </c>
+      <c r="J172" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>46.61</v>
+      </c>
+      <c r="B173">
+        <v>23.44</v>
+      </c>
       <c r="C173">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>46.61</v>
+      </c>
+      <c r="D173">
+        <v>21.93</v>
+      </c>
+      <c r="E173">
+        <v>47.25</v>
       </c>
       <c r="F173">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G173">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>47.25</v>
       </c>
       <c r="H173">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.35">
+        <v>23.44</v>
+      </c>
+      <c r="I173">
+        <v>6.1</v>
+      </c>
+      <c r="J173" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>47.25</v>
+      </c>
+      <c r="B174">
+        <v>24.65</v>
+      </c>
       <c r="C174">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>47.25</v>
+      </c>
+      <c r="D174">
+        <v>21.93</v>
+      </c>
+      <c r="E174">
+        <v>48.03</v>
       </c>
       <c r="F174">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G174">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>48.03</v>
       </c>
       <c r="H174">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I174">
+        <v>6.1</v>
+      </c>
+      <c r="J174" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>48.03</v>
+      </c>
+      <c r="B175">
+        <v>24.65</v>
+      </c>
       <c r="C175">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>48.03</v>
+      </c>
+      <c r="D175">
+        <v>21.93</v>
+      </c>
+      <c r="E175">
+        <v>48.74</v>
       </c>
       <c r="F175">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G175">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>48.74</v>
       </c>
       <c r="H175">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I175">
+        <v>6.1</v>
+      </c>
+      <c r="J175" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>48.16</v>
+      </c>
+      <c r="B176">
+        <v>24.65</v>
+      </c>
       <c r="C176">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>48.16</v>
+      </c>
+      <c r="D176">
+        <v>24.59</v>
+      </c>
+      <c r="E176">
+        <v>48.61</v>
       </c>
       <c r="F176">
-        <f t="shared" si="29"/>
-        <v>0</v>
+        <f>D176</f>
+        <v>24.59</v>
       </c>
       <c r="G176">
-        <f t="shared" si="30"/>
-        <v>0</v>
+        <f>E176</f>
+        <v>48.61</v>
       </c>
       <c r="H176">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="177" spans="3:8" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I176">
+        <v>6.1</v>
+      </c>
+      <c r="J176" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>48.74</v>
+      </c>
+      <c r="B177">
+        <v>24.65</v>
+      </c>
       <c r="C177">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>48.74</v>
+      </c>
+      <c r="D177">
+        <v>24.39</v>
+      </c>
+      <c r="E177">
+        <v>49.42</v>
       </c>
       <c r="F177">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>24.39</v>
       </c>
       <c r="G177">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>49.42</v>
       </c>
       <c r="H177">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="178" spans="3:8" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I177">
+        <v>6.1</v>
+      </c>
+      <c r="J177" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>48.74</v>
+      </c>
+      <c r="B178">
+        <v>24.39</v>
+      </c>
       <c r="C178">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>48.74</v>
+      </c>
+      <c r="D178">
+        <v>24.01</v>
+      </c>
+      <c r="E178">
+        <v>49.42</v>
       </c>
       <c r="F178">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>24.01</v>
       </c>
       <c r="G178">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>49.42</v>
       </c>
       <c r="H178">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="179" spans="3:8" x14ac:dyDescent="0.35">
+        <v>24.39</v>
+      </c>
+      <c r="I178">
+        <v>6.1</v>
+      </c>
+      <c r="J178" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>48.74</v>
+      </c>
+      <c r="B179">
+        <v>24.01</v>
+      </c>
       <c r="C179">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>48.74</v>
+      </c>
+      <c r="D179">
+        <v>23.69</v>
+      </c>
+      <c r="E179">
+        <v>49.42</v>
       </c>
       <c r="F179">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>23.69</v>
       </c>
       <c r="G179">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>49.42</v>
       </c>
       <c r="H179">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="180" spans="3:8" x14ac:dyDescent="0.35">
+        <v>24.01</v>
+      </c>
+      <c r="I179">
+        <v>6.1</v>
+      </c>
+      <c r="J179" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>48.74</v>
+      </c>
+      <c r="B180">
+        <v>23.69</v>
+      </c>
       <c r="C180">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>48.74</v>
+      </c>
+      <c r="D180">
+        <v>21.93</v>
+      </c>
+      <c r="E180">
+        <v>49.42</v>
       </c>
       <c r="F180">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G180">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>49.42</v>
       </c>
       <c r="H180">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="181" spans="3:8" x14ac:dyDescent="0.35">
+        <v>23.69</v>
+      </c>
+      <c r="I180">
+        <v>6.1</v>
+      </c>
+      <c r="J180" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>49.42</v>
+      </c>
+      <c r="B181">
+        <v>24.65</v>
+      </c>
       <c r="C181">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>49.42</v>
+      </c>
+      <c r="D181">
+        <v>22.61</v>
+      </c>
+      <c r="E181">
+        <v>50.13</v>
       </c>
       <c r="F181">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>22.61</v>
       </c>
       <c r="G181">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>50.13</v>
       </c>
       <c r="H181">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="182" spans="3:8" x14ac:dyDescent="0.35">
+        <v>24.65</v>
+      </c>
+      <c r="I181">
+        <v>6.1</v>
+      </c>
+      <c r="J181" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>49.42</v>
+      </c>
+      <c r="B182">
+        <v>22.61</v>
+      </c>
       <c r="C182">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>49.42</v>
+      </c>
+      <c r="D182">
+        <v>21.93</v>
+      </c>
+      <c r="E182">
+        <v>50.13</v>
       </c>
       <c r="F182">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>21.93</v>
       </c>
       <c r="G182">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>50.13</v>
       </c>
       <c r="H182">
         <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="183" spans="3:8" x14ac:dyDescent="0.35">
+        <v>22.61</v>
+      </c>
+      <c r="I182">
+        <v>6.1</v>
+      </c>
+      <c r="J182" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>50.13</v>
+      </c>
+      <c r="B183">
+        <v>24.65</v>
+      </c>
       <c r="C183">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>50.13</v>
+      </c>
+      <c r="D183">
+        <v>23.3</v>
+      </c>
+      <c r="E183">
+        <v>50.89</v>
       </c>
       <c r="F183">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>23.3</v>
       </c>
       <c r="G183">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>50.89</v>
       </c>
       <c r="H183">
         <f t="shared" si="31"/>
+        <v>24.65</v>
+      </c>
+      <c r="I183">
+        <v>6.1</v>
+      </c>
+      <c r="J183" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>50.13</v>
+      </c>
+      <c r="B184">
+        <v>23.3</v>
+      </c>
+      <c r="C184">
+        <f t="shared" ref="C184:C200" si="32">A184</f>
+        <v>50.13</v>
+      </c>
+      <c r="D184">
+        <v>21.93</v>
+      </c>
+      <c r="E184">
+        <v>50.89</v>
+      </c>
+      <c r="F184">
+        <f t="shared" ref="F184:F200" si="33">D184</f>
+        <v>21.93</v>
+      </c>
+      <c r="G184">
+        <f t="shared" ref="G184:G200" si="34">E184</f>
+        <v>50.89</v>
+      </c>
+      <c r="H184">
+        <f t="shared" ref="H184:H200" si="35">B184</f>
+        <v>23.3</v>
+      </c>
+      <c r="I184">
+        <v>6.1</v>
+      </c>
+      <c r="J184" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>50.89</v>
+      </c>
+      <c r="B185">
+        <v>24.65</v>
+      </c>
+      <c r="C185">
+        <f t="shared" si="32"/>
+        <v>50.89</v>
+      </c>
+      <c r="D185">
+        <v>24.35</v>
+      </c>
+      <c r="E185">
+        <v>51.64</v>
+      </c>
+      <c r="F185">
+        <f t="shared" si="33"/>
+        <v>24.35</v>
+      </c>
+      <c r="G185">
+        <f t="shared" si="34"/>
+        <v>51.64</v>
+      </c>
+      <c r="H185">
+        <f t="shared" si="35"/>
+        <v>24.65</v>
+      </c>
+      <c r="I185">
+        <v>6.1</v>
+      </c>
+      <c r="J185" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>50.89</v>
+      </c>
+      <c r="B186">
+        <v>24.35</v>
+      </c>
+      <c r="C186">
+        <f t="shared" si="32"/>
+        <v>50.89</v>
+      </c>
+      <c r="D186">
+        <v>21.93</v>
+      </c>
+      <c r="E186">
+        <v>51.64</v>
+      </c>
+      <c r="F186">
+        <f t="shared" si="33"/>
+        <v>21.93</v>
+      </c>
+      <c r="G186">
+        <f t="shared" si="34"/>
+        <v>51.64</v>
+      </c>
+      <c r="H186">
+        <f t="shared" si="35"/>
+        <v>24.35</v>
+      </c>
+      <c r="I186">
+        <v>6.1</v>
+      </c>
+      <c r="J186" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C187">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F187">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G187">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H187">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C188">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F188">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G188">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H188">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C189">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F189">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G189">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H189">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C190">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F190">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G190">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H190">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C191">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F191">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G191">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H191">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C192">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F192">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G192">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H192">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C193">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F193">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G193">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H193">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C194">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F194">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G194">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H194">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C195">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F195">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G195">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H195">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C196">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F196">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G196">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H196">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C197">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F197">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G197">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H197">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C198">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F198">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G198">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H198">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C199">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F199">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G199">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H199">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C200">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="F200">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="G200">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="H200">
+        <f t="shared" si="35"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>